<commit_message>
feat(figures): update Figure 3 to all 17 clinical concept categories and backup 10-category script
</commit_message>
<xml_diff>
--- a/publication/results/tables/table4_category_breakdown_faers.xlsx
+++ b/publication/results/tables/table4_category_breakdown_faers.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESM_Cover_Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_4_Category_Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_4_17_Categories" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Table 4: FAERS Per-Category Performance Breakdown</t>
+          <t>Table 4: FAERS 17-Category Performance Breakdown</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Two-Tier Evaluation Framework (Tier 1: Strict CoNLL; Tier 2: Adapted ADE-Eval)</t>
+          <t>Two-Tier Evaluation Framework across all 17 clinical concept categories</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,647 +535,757 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Gold Support (N)</t>
+          <t>Gold_N</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>BioBERT LOO Strict F1</t>
+          <t>BioBERT_Strict</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>BioBERT LOO ADE-Eval F1</t>
+          <t>LLaMA4_Strict</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Claude Sonnet Strict F1</t>
+          <t>Sonnet_Strict</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Claude Sonnet ADE-Eval F1</t>
+          <t>BioBERT_ADE</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>LLaMA 4 (Tagged) Strict F1</t>
+          <t>LLaMA4_ADE</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LLaMA 4 (Tagged) ADE-Eval F1</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>LLaMA 4 (JSON) Strict F1</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>LLaMA 4 (JSON) ADE-Eval F1</t>
+          <t>Sonnet_ADE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>sDrug</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9186</v>
+        <v>4665</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$0.5115 \pm 0.0476$</t>
+          <t>0.6025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>$0.6966 \pm 0.0415$</t>
+          <t>0.3181</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.4609</t>
+          <t>0.4006</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.6259</t>
+          <t>0.7376</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.4320</t>
+          <t>0.5463</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.6508</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.4306</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.6048</t>
+          <t>0.5619</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>cDrug</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>787</v>
+        <v>2995</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$0.9173 \pm 0.0597$</t>
+          <t>0.7433</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>$0.9492 \pm 0.0344$</t>
+          <t>0.3443</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.8873</t>
+          <t>0.5689</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.9305</t>
+          <t>0.8451</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.8303</t>
+          <t>0.6013</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.9203</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.8281</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.9165</t>
+          <t>0.7130</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>oDrug</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.0171</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.4605</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.0106</t>
+          <t>0.4804</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.4687</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.4370</t>
+          <t>0.4848</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DOSE</t>
+          <t>Dose</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1619</v>
+        <v>1668</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>$0.4666 \pm 0.0645$</t>
+          <t>0.6100</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>$0.6972 \pm 0.0370$</t>
+          <t>0.2752</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.4436</t>
+          <t>0.4300</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.6944</t>
+          <t>0.7427</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.3776</t>
+          <t>0.5783</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.6492</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.2126</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>0.5836</t>
+          <t>0.6826</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DRUG</t>
+          <t>Indication</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6673</v>
+        <v>202</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$0.5280 \pm 0.0730$</t>
+          <t>0.1335</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$0.7156 \pm 0.0445$</t>
+          <t>0.0690</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.4528</t>
+          <t>0.1042</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.6379</t>
+          <t>0.5021</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.3816</t>
+          <t>0.4913</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.6222</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.4163</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>0.6141</t>
+          <t>0.5194</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1543</v>
+        <v>1490</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$0.4253 \pm 0.0556$</t>
+          <t>0.6260</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$0.6599 \pm 0.0486$</t>
+          <t>0.1832</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.2621</t>
+          <t>0.3189</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.5159</t>
+          <t>0.7775</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.2170</t>
+          <t>0.4647</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.5073</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.1910</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>0.4964</t>
+          <t>0.5355</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HX</t>
+          <t>AE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2408</v>
+        <v>12010</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$0.6099 \pm 0.1357$</t>
+          <t>0.5931</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>$0.7875 \pm 0.0928$</t>
+          <t>0.3582</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.5526</t>
+          <t>0.4401</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.7165</t>
+          <t>0.7066</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.4568</t>
+          <t>0.5635</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0.6672</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.4664</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>0.6481</t>
+          <t>0.5678</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INDICATION</t>
+          <t>mAE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>162</v>
+        <v>113</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>$0.0368 \pm 0.0470$</t>
+          <t>0.0480</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>$0.0864 \pm 0.1080$</t>
+          <t>0.0405</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.1178</t>
+          <t>0.0594</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.4617</t>
+          <t>0.0507</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.1074</t>
+          <t>0.4604</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.4493</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.0866</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>0.4355</t>
+          <t>0.4574</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>Dx</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3476</v>
+        <v>64</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>$0.4519 \pm 0.0945$</t>
+          <t>0.0670</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>$0.6743 \pm 0.0649$</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.3623</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.6143</t>
+          <t>0.4536</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.2225</t>
+          <t>0.4016</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.5549</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.2006</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>0.5134</t>
+          <t>0.3704</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>Lab</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>3482</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.5964</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.1575</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.0144</t>
+          <t>0.3742</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.4512</t>
+          <t>0.7637</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.0074</t>
+          <t>0.4912</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0.4466</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.0370</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>0.4731</t>
+          <t>0.6105</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SEX</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>767</v>
+        <v>1910</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>$0.9213 \pm 0.0189$</t>
+          <t>0.7169</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>$0.9571 \pm 0.0225$</t>
+          <t>0.1304</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.8922</t>
+          <t>0.2741</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.9449</t>
+          <t>0.8386</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.8269</t>
+          <t>0.2676</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.9078</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.7928</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>0.8957</t>
+          <t>0.4547</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>R/O</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1796</v>
+        <v>9</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>$0.6112 \pm 0.1034$</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$0.7575 \pm 0.0864$</t>
+          <t>0.0073</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.2896</t>
+          <t>0.0094</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.4663</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.1908</t>
+          <t>0.4444</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.3072</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.2636</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>0.4753</t>
+          <t>0.4539</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.0052</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0.0165</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.4610</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.4686</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MHx</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2370</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.4621</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.3474</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.4896</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.7138</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.6121</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.6888</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FHx</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>105</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.0727</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.0606</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.1395</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0818</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.1736</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.2130</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>787</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.9009</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.7335</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.8752</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.9525</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.8590</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.9238</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>777</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.9037</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.7551</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.8829</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.9570</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.8575</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.9376</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>32650</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.6032</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.2982</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.4189</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.7477</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.5515</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.6060</t>
         </is>
       </c>
     </row>

</xml_diff>